<commit_message>
Muitas atualizações - foi mal time muito tempo sem dar update entao nem sei o que mudou so sei que tem BI, contagem etc etc.. analise os arquivos pra saber mais (aloca)
</commit_message>
<xml_diff>
--- a/GTSEGURANCA_gerador_graficos/Okuhara_e_outras_regioes/regioes.xlsx
+++ b/GTSEGURANCA_gerador_graficos/Okuhara_e_outras_regioes/regioes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\x387162\Desktop\Relatorio_Diario\GTSEGURANCA_gerador_graficos\Okuhara_e_outras_regioes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B89A090D-F717-4F2D-8A5A-F25D956777A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5787DF1-74E8-40D7-AFCB-6BCA0FEF6CEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,27 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$91</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="116">
   <si>
     <t>Original</t>
   </si>
@@ -127,9 +140,6 @@
     <t>Parque Dom Pedro II - Viaduto Antônio Nakashima (embaixo do viaduto/quadrado)</t>
   </si>
   <si>
-    <t>Parque Dom Pedro II - Viaduto Antônio Nakashima</t>
-  </si>
-  <si>
     <t>Parque Dom Pedro II</t>
   </si>
   <si>
@@ -358,7 +368,22 @@
     <t>Complexo Okuhara Koei - Rua Major Natanael (ao lado do Cemitério da Consolação)</t>
   </si>
   <si>
-    <t>Viaduto Antônio Nakashima x Viaduto Vinte e Cinco de Março</t>
+    <t>Avenida Rangel Pestana, 267/Travessa da Rua da Figueira 274/Triangulo</t>
+  </si>
+  <si>
+    <t>Praça Roosevelt - Embaixo do viaduto</t>
+  </si>
+  <si>
+    <t>Praça Roosevelt</t>
+  </si>
+  <si>
+    <t>Praça Ragueb Chohfi</t>
+  </si>
+  <si>
+    <t>Viaduto Antônio Nakashima (embaixo do viaduto, próximo a escola)</t>
+  </si>
+  <si>
+    <t>Itapura de Miranda embaixo da alça viaduto Diário Popular</t>
   </si>
 </sst>
 </file>
@@ -721,7 +746,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C89"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="116.140625" bestFit="1" customWidth="1"/>
@@ -740,62 +766,62 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" t="s">
         <v>40</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" t="s">
         <v>40</v>
       </c>
-      <c r="C2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>70</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B6" t="s">
         <v>70</v>
       </c>
-      <c r="C4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="C6" t="s">
         <v>68</v>
       </c>
-      <c r="B5" t="s">
-        <v>68</v>
-      </c>
-      <c r="C5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" t="s">
-        <v>71</v>
-      </c>
-      <c r="C6" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -806,7 +832,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -817,7 +843,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -828,7 +854,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -839,40 +865,40 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" t="s">
         <v>46</v>
       </c>
-      <c r="B11" t="s">
+    </row>
+    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" t="s">
         <v>46</v>
       </c>
-      <c r="C11" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    </row>
+    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>48</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
         <v>48</v>
       </c>
-      <c r="C12" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" t="s">
-        <v>49</v>
-      </c>
       <c r="C13" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -883,7 +909,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -894,7 +920,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -905,40 +931,40 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C17" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>85</v>
-      </c>
       <c r="B18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C18" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>82</v>
+      </c>
+      <c r="B19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" t="s">
         <v>83</v>
       </c>
-      <c r="B19" t="s">
-        <v>83</v>
-      </c>
-      <c r="C19" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -949,18 +975,18 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21" t="s">
         <v>38</v>
       </c>
-      <c r="B21" t="s">
-        <v>38</v>
-      </c>
-      <c r="C21" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>15</v>
       </c>
@@ -968,10 +994,10 @@
         <v>15</v>
       </c>
       <c r="C22" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>3</v>
       </c>
@@ -982,7 +1008,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>10</v>
       </c>
@@ -993,7 +1019,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>11</v>
       </c>
@@ -1004,7 +1030,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -1015,7 +1041,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>13</v>
       </c>
@@ -1026,18 +1052,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>9</v>
       </c>
       <c r="B28" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C28" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>16</v>
       </c>
@@ -1045,21 +1071,21 @@
         <v>16</v>
       </c>
       <c r="C29" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B30" t="s">
         <v>16</v>
       </c>
       <c r="C30" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>17</v>
       </c>
@@ -1067,87 +1093,87 @@
         <v>16</v>
       </c>
       <c r="C31" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C32" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B33" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C33" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B34" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C34" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B35" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C35" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B36" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C36" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B37" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C37" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B38" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C38" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>26</v>
       </c>
@@ -1158,9 +1184,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B40" t="s">
         <v>27</v>
@@ -1169,9 +1195,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B41" t="s">
         <v>27</v>
@@ -1180,73 +1206,73 @@
         <v>28</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>94</v>
+      </c>
+      <c r="B42" t="s">
         <v>95</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>99</v>
+      </c>
+      <c r="B43" t="s">
+        <v>95</v>
+      </c>
+      <c r="C43" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>100</v>
+      </c>
+      <c r="B44" t="s">
+        <v>95</v>
+      </c>
+      <c r="C44" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>91</v>
+      </c>
+      <c r="B45" t="s">
+        <v>91</v>
+      </c>
+      <c r="C45" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>92</v>
+      </c>
+      <c r="B46" t="s">
+        <v>92</v>
+      </c>
+      <c r="C46" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>96</v>
       </c>
-      <c r="C42" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>100</v>
-      </c>
-      <c r="B43" t="s">
+      <c r="B47" t="s">
         <v>96</v>
       </c>
-      <c r="C43" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>101</v>
-      </c>
-      <c r="B44" t="s">
-        <v>96</v>
-      </c>
-      <c r="C44" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>92</v>
-      </c>
-      <c r="B45" t="s">
-        <v>92</v>
-      </c>
-      <c r="C45" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>93</v>
-      </c>
-      <c r="B46" t="s">
-        <v>93</v>
-      </c>
-      <c r="C46" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>97</v>
-      </c>
-      <c r="B47" t="s">
-        <v>97</v>
-      </c>
       <c r="C47" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>29</v>
       </c>
@@ -1257,9 +1283,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B49" t="s">
         <v>30</v>
@@ -1268,7 +1294,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>32</v>
       </c>
@@ -1279,9 +1305,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B51" t="s">
         <v>32</v>
@@ -1290,9 +1316,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B52" t="s">
         <v>32</v>
@@ -1301,224 +1327,224 @@
         <v>28</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B53" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C53" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>42</v>
+      </c>
+      <c r="B54" t="s">
+        <v>42</v>
+      </c>
+      <c r="C54" t="s">
         <v>43</v>
       </c>
-      <c r="B54" t="s">
-        <v>43</v>
-      </c>
-      <c r="C54" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>60</v>
+      </c>
+      <c r="B55" t="s">
+        <v>60</v>
+      </c>
+      <c r="C55" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" t="s">
+        <v>58</v>
+      </c>
+      <c r="C56" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>63</v>
+      </c>
+      <c r="B57" t="s">
+        <v>63</v>
+      </c>
+      <c r="C57" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>49</v>
+      </c>
+      <c r="B58" t="s">
+        <v>49</v>
+      </c>
+      <c r="C58" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>65</v>
+      </c>
+      <c r="B59" t="s">
+        <v>65</v>
+      </c>
+      <c r="C59" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>52</v>
+      </c>
+      <c r="B60" t="s">
+        <v>52</v>
+      </c>
+      <c r="C60" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>57</v>
+      </c>
+      <c r="B61" t="s">
+        <v>57</v>
+      </c>
+      <c r="C61" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>54</v>
+      </c>
+      <c r="B62" t="s">
+        <v>54</v>
+      </c>
+      <c r="C62" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>51</v>
+      </c>
+      <c r="B63" t="s">
+        <v>51</v>
+      </c>
+      <c r="C63" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>64</v>
+      </c>
+      <c r="B64" t="s">
+        <v>64</v>
+      </c>
+      <c r="C64" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
         <v>61</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B65" t="s">
         <v>61</v>
       </c>
-      <c r="C55" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+      <c r="C65" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>56</v>
+      </c>
+      <c r="B66" t="s">
+        <v>56</v>
+      </c>
+      <c r="C66" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>55</v>
+      </c>
+      <c r="B67" t="s">
+        <v>55</v>
+      </c>
+      <c r="C67" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>62</v>
+      </c>
+      <c r="B68" t="s">
+        <v>62</v>
+      </c>
+      <c r="C68" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>53</v>
+      </c>
+      <c r="B69" t="s">
+        <v>53</v>
+      </c>
+      <c r="C69" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
         <v>59</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B70" t="s">
         <v>59</v>
       </c>
-      <c r="C56" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>64</v>
-      </c>
-      <c r="B57" t="s">
-        <v>64</v>
-      </c>
-      <c r="C57" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+      <c r="C70" t="s">
         <v>50</v>
       </c>
-      <c r="B58" t="s">
+    </row>
+    <row r="71" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>66</v>
+      </c>
+      <c r="B71" t="s">
+        <v>66</v>
+      </c>
+      <c r="C71" t="s">
         <v>50</v>
-      </c>
-      <c r="C58" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>66</v>
-      </c>
-      <c r="B59" t="s">
-        <v>66</v>
-      </c>
-      <c r="C59" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>53</v>
-      </c>
-      <c r="B60" t="s">
-        <v>53</v>
-      </c>
-      <c r="C60" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>58</v>
-      </c>
-      <c r="B61" t="s">
-        <v>58</v>
-      </c>
-      <c r="C61" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>55</v>
-      </c>
-      <c r="B62" t="s">
-        <v>55</v>
-      </c>
-      <c r="C62" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>52</v>
-      </c>
-      <c r="B63" t="s">
-        <v>52</v>
-      </c>
-      <c r="C63" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>65</v>
-      </c>
-      <c r="B64" t="s">
-        <v>65</v>
-      </c>
-      <c r="C64" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>62</v>
-      </c>
-      <c r="B65" t="s">
-        <v>62</v>
-      </c>
-      <c r="C65" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>57</v>
-      </c>
-      <c r="B66" t="s">
-        <v>57</v>
-      </c>
-      <c r="C66" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>56</v>
-      </c>
-      <c r="B67" t="s">
-        <v>56</v>
-      </c>
-      <c r="C67" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>63</v>
-      </c>
-      <c r="B68" t="s">
-        <v>63</v>
-      </c>
-      <c r="C68" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>54</v>
-      </c>
-      <c r="B69" t="s">
-        <v>54</v>
-      </c>
-      <c r="C69" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>60</v>
-      </c>
-      <c r="B70" t="s">
-        <v>60</v>
-      </c>
-      <c r="C70" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>67</v>
-      </c>
-      <c r="B71" t="s">
-        <v>67</v>
-      </c>
-      <c r="C71" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B72" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C72" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
@@ -1526,21 +1552,21 @@
         <v>33</v>
       </c>
       <c r="B73" t="s">
+        <v>114</v>
+      </c>
+      <c r="C73" t="s">
         <v>34</v>
-      </c>
-      <c r="C73" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B74" t="s">
+        <v>114</v>
+      </c>
+      <c r="C74" t="s">
         <v>34</v>
-      </c>
-      <c r="C74" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
@@ -1548,168 +1574,203 @@
         <v>33</v>
       </c>
       <c r="B75" t="s">
+        <v>114</v>
+      </c>
+      <c r="C75" t="s">
         <v>34</v>
       </c>
-      <c r="C75" t="s">
+    </row>
+    <row r="76" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+      <c r="B76" t="s">
+        <v>35</v>
+      </c>
+      <c r="C76" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>36</v>
       </c>
-      <c r="B76" t="s">
-        <v>36</v>
-      </c>
-      <c r="C76" t="s">
+      <c r="B77" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>37</v>
-      </c>
-      <c r="B77" t="s">
-        <v>36</v>
-      </c>
       <c r="C77" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>89</v>
+      </c>
+      <c r="B78" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>90</v>
-      </c>
-      <c r="B78" t="s">
-        <v>36</v>
-      </c>
       <c r="C78" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B79" t="s">
-        <v>89</v>
+        <v>113</v>
       </c>
       <c r="C79" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>75</v>
+      </c>
+      <c r="B80" t="s">
+        <v>75</v>
+      </c>
+      <c r="C80" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
         <v>76</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B81" t="s">
         <v>76</v>
       </c>
-      <c r="C80" t="s">
+      <c r="C81" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>77</v>
+      </c>
+      <c r="B82" t="s">
+        <v>77</v>
+      </c>
+      <c r="C82" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>77</v>
-      </c>
-      <c r="B81" t="s">
-        <v>77</v>
-      </c>
-      <c r="C81" t="s">
+      <c r="B83" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
+      <c r="C83" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>71</v>
+      </c>
+      <c r="B84" t="s">
+        <v>71</v>
+      </c>
+      <c r="C84" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>74</v>
+      </c>
+      <c r="B85" t="s">
+        <v>74</v>
+      </c>
+      <c r="C85" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>80</v>
+      </c>
+      <c r="B86" t="s">
+        <v>80</v>
+      </c>
+      <c r="C86" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>81</v>
+      </c>
+      <c r="B87" t="s">
+        <v>81</v>
+      </c>
+      <c r="C87" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>78</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B88" t="s">
         <v>78</v>
       </c>
-      <c r="C82" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>74</v>
-      </c>
-      <c r="B83" t="s">
-        <v>74</v>
-      </c>
-      <c r="C83" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>72</v>
-      </c>
-      <c r="B84" t="s">
-        <v>72</v>
-      </c>
-      <c r="C84" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>75</v>
-      </c>
-      <c r="B85" t="s">
-        <v>75</v>
-      </c>
-      <c r="C85" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>81</v>
-      </c>
-      <c r="B86" t="s">
-        <v>81</v>
-      </c>
-      <c r="C86" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>82</v>
-      </c>
-      <c r="B87" t="s">
-        <v>82</v>
-      </c>
-      <c r="C87" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
+      <c r="C88" t="s">
         <v>79</v>
       </c>
-      <c r="B88" t="s">
-        <v>79</v>
-      </c>
-      <c r="C88" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="89" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>109</v>
+      </c>
+      <c r="B89" t="s">
+        <v>109</v>
+      </c>
+      <c r="C89" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>110</v>
       </c>
-      <c r="B89" t="s">
-        <v>110</v>
-      </c>
-      <c r="C89" t="s">
-        <v>109</v>
+      <c r="B90" t="s">
+        <v>115</v>
+      </c>
+      <c r="C90" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>111</v>
+      </c>
+      <c r="B91" t="s">
+        <v>24</v>
+      </c>
+      <c r="C91" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C88" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="A1:C91" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Parque Dom Pedro II - Viaduto Antônio Nakashima"/>
+        <filter val="Viaduto Antônio Nakashima x Viaduto Vinte e Cinco de Março"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Complexo Okuhara Koei"/>
+        <filter val="Glicério"/>
+        <filter val="Parque Dom Pedro II"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C88">
       <sortCondition ref="C1:C88"/>
     </sortState>

</xml_diff>